<commit_message>
Finish excel-driven testcases for INS, static, and study listing across apps
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/C3DC_StaticData.xlsx
+++ b/InputFiles/C3DC/C3DC_StaticData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12820" yWindow="-27140" windowWidth="31900" windowHeight="18140" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12820" yWindow="-27140" windowWidth="31900" windowHeight="18140" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HomePage" sheetId="1" state="visible" r:id="rId1"/>
@@ -646,7 +646,7 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>/release-notes-pdf</t>
+          <t>/release_notes_pdf</t>
         </is>
       </c>
     </row>

</xml_diff>